<commit_message>
feat: update 9988.HK and BABA for Q1 FY2027 and the August placing
Adds the June Quarter 2026 results (6-K EX-99.1, 2026-08-20) to both
lines and rebuilds one shared RMB-level owner-FCF model. The 710M-share
HK$112.70 placing completed 2026-08-26 is added to the share count and
its net proceeds to cash. Weighted IV: 9988.HK HK$93.31 -> 91.50,
BABA US$126.35 -> 93.33 per ADS.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/research/9988.HK/Reports/9988.HK_DCF_Model.xlsx
+++ b/research/9988.HK/Reports/9988.HK_DCF_Model.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="199">
   <si>
     <t xml:space="preserve">Ticker</t>
   </si>
@@ -53,13 +53,13 @@
     <t xml:space="preserve">Price as of</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-10-21T08:08:18Z HKEX regular close</t>
+    <t xml:space="preserve">2026-10-22T01:20:45Z HKEX morning session (intraday print, not a close; replace at the next regular close)</t>
   </si>
   <si>
     <t xml:space="preserve">Balance sheet date</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-03-31</t>
+    <t xml:space="preserve">2026-06-30</t>
   </si>
   <si>
     <t xml:space="preserve">Model</t>
@@ -95,7 +95,7 @@
     <t xml:space="preserve">Built at</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-10-22T01:02:13Z</t>
+    <t xml:space="preserve">2026-10-22T01:44:36Z</t>
   </si>
   <si>
     <t xml:space="preserve">Drivers file</t>
@@ -113,34 +113,34 @@
     <t xml:space="preserve">Methodology</t>
   </si>
   <si>
-    <t xml:space="preserve">summary: FY2026-FY2029 are investment-trough years by choice, not demand decline, but the July 2026 build normalised that trough away by starting from a mid-cycle RMB120bn FCF. The Q1 FY2027 print (capex RMB67.7bn, FCF -44.7bn, buybacks -80%, AI Labs -13.9bn, CMR -7% reported) showed the trough deepening in year 1 rather than recovering, so this build models the capex supercycle explicitly as a component owner-FCF path with negative FCF through FY2029 and the recovery pushed to FY2030, discounted at a single RMB-built 10% WACC that carries a widened regulatory/litigation premium for the EU DSA exposure and the DoD designation. Terminal value is Gordon-bound in base and bear (implied ~6x EV/EBITDA, below the FY2022-25 normal-year 8.1x average), so no multiple expansion is assumed; the strategic investment portfolio (Ant etc.) enters the bridge at half book and NCI is deducted, both for the first time. The buyback cut does not change the flat share count (SBC is expensed in full, so buybacks are value-neutral here) but it removes a price support the market had been leaning on, which is reflected in the weights, not the flows.
-key_risks_to_valuation: Capex intensity: every 1pp of FY2027-FY2031 capex/revenue that does not normalise is ~RMB 60-70bn of cumulative owner FCF; the base assumes intensity halves from 22% to 11% by FY2032.; Cloud deceleration below 30% before margin matures would break the base margin path (22% mature EBITDA).; EU DSA follow-on penalties (up to 6% of global turnover) and a DoD 1260H loss are in the discount rate (1.25pp), not the flows; a realised penalty of that size would be a flow event.; Investment-portfolio bridge (HK$13.7/share at 50% of book) depends on Ant Group's realisable value and PRC exit taxes; strike it and the weighted IV falls by that amount.; RMB/HKD: every 1% move in CNYHKD moves every HKD value 1%; fx_rate is dated 2026-10-22 and is not refreshed by refresh_price.py.; Mainland Southbound flows are a 9988.HK-specific demand source that can move the HK price away from the ADS parity line for extended periods; the valuation ignores it.</t>
+    <t xml:space="preserve">summary: FY2026-FY2029 are investment-trough years by choice, not demand decline. This build models the capex supercycle explicitly as a component owner-FCF path with negative FCF through FY2029 and the recovery pushed to FY2030, discounted at a single RMB-built 10% WACC that carries a regulatory/litigation premium for the EU DSA exposure and the DoD designation. Versus this morning's version the anchors move to the 30 Jun 2026 balance sheet (net cash down RMB53bn in the quarter) and the 26 Aug 2026 placing (710M shares, RMB ~68bn), with the Q1 burn charged once via a stub add-back and the July dividend deducted; FY2027-28 capex intensity is 1pp higher and SBC is held at a 1.3% plateau. Terminal value is Gordon-bound in base (implied ~6x EV/EBITDA, below the FY2022-25 normal-year 8.1x average), so no multiple expansion is assumed; the strategic investment portfolio (Ant etc.) enters the bridge at half book and NCI is deducted. The placing is the fact that matters most for how to read the stock: a company that was the market's largest buyer of its own shares in FY2024-25 is now a net issuer, at a price near the bottom of its 52-week range, to fund compute. That is reflected in the share count and cash, and in the capex path -- not in the weights, which were already moved toward the bear this morning.
+key_risks_to_valuation: Capex intensity: every 1pp of FY2027-FY2031 capex/revenue that does not normalise is ~RMB 60-70bn of cumulative owner FCF; the base assumes intensity halves from 23% to 11% by FY2032. The placing shows the company is willing to fund overshoot with equity, which dilutes rather than merely burns.; Cloud deceleration below 30% before margin matures would break the base margin path (22% mature EBITDA).; EU DSA follow-on penalties (up to 6% of global turnover) and a DoD 1260H loss are in the discount rate (1.25pp), not the flows; a realised penalty of that size would be a flow event.; Investment-portfolio bridge (~HK$13.3/share at 50% of book) depends on Ant Group's realisable value and PRC exit taxes; strike it and the weighted IV falls by that amount.; RMB/HKD: every 1% move in CNYHKD moves every HKD value 1%; fx_rate is dated 2026-10-22 and is not refreshed by refresh_price.py. The placing proceeds are also converted at that rate.; Further equity issuance: a second placing of similar size at a price below IV would be dilutive; the model assumes the count is flat at 20,034M from here.; Mainland Southbound flows are a 9988.HK-specific demand source that can move the HK price away from the ADS parity line for extended periods; the valuation ignores it.</t>
   </si>
   <si>
     <t xml:space="preserve">Data sources</t>
   </si>
   <si>
-    <t xml:space="preserve">price: Yahoo Finance chart API at inputs.price_as_of (HKEX regular close); 52-week range HK$88.65-175.00. BABA ADS parity check in inputs.fx_note.
-financials: 9988.HK_Metrics.csv (unchanged, FY2026 latest annual, RMB millions, derived from the FY2026 20-F iXBRL extract 9988.HK_Annual_FY2026.txt); component lines cited by file:line in inputs.* and equity_bridge.*. Q1 FY2027 (20 Aug 2026) figures are taken from 9988.HK_Analysis.json; that release is not extracted.
+    <t xml:space="preserve">price: Yahoo Finance chart API at inputs.price_as_of (HKEX intraday, morning session); 52-week range HK$88.65-175.00. BABA ADS parity check in inputs.fx_note.
+financials: 9988.HK_Metrics.csv (FY2026 latest annual plus the new Q1 FY2027 row, RMB millions). Q1 FY2027 balance sheet, segment tables, SBC, capex and FCF read from 9988.HK_Quarterly_Q1-FY2027.txt (results announcement for the quarter ended 30 Jun 2026, released 20 Aug 2026), cited by line in inputs.* and equity_bridge.*. FY0 flows from the FY2026 20-F (9988.HK_Annual_FY2026.txt). Placing: Alibaba 6-K filed 2026-08-26 (accession 0001193125-26-365894), figures supplied by the orchestrator; the ShortTermInvestments/OtherTreasuryInvestments cells for the Q1 row are taken from release line 707 because the CSV export leaves them blank.
 qualitative: 9988.HK_Analysis.json (analysis_date 2026-10-22).</t>
   </si>
   <si>
     <t xml:space="preserve">Scenario narrative: bear</t>
   </si>
   <si>
-    <t xml:space="preserve">The capex supercycle does not pay: management keeps spending through FY2028 (RMB ~500bn over two years) into a price-competitive China AI market (DeepSeek, ByteDance, Huawei), cloud growth decelerates below 25%, AI Labs keeps burning, and the capex is cut only after the returns disappoint. Quick-commerce breakeven slips as Meituan re-engages; CMR resumes low-single-digit decline. On the regulatory axis the EU judges AliExpress remediation inadequate and levies follow-on DSA penalties, and the DoD designation survives the Northern District of California challenge, keeping US institutions out. Owner FCF stays negative until FY2031 and the business is worth little more than its balance sheet (net cash + investments ~HK$26/share of the ~HK$51 bear value).</t>
+    <t xml:space="preserve">The capex supercycle does not pay: management keeps spending through FY2028 (RMB ~520bn over two years, part of it the August 2026 equity) into a price-competitive China AI market (DeepSeek, ByteDance, Huawei), cloud growth decelerates below 25%, AI Labs keeps burning, and the capex is cut only after the returns disappoint. Quick-commerce breakeven slips as Meituan re-engages; CMR resumes low-single-digit decline. On the regulatory axis the EU judges AliExpress remediation inadequate and levies follow-on DSA penalties, and the DoD designation survives the Northern District of California challenge, keeping US institutions out. Owner FCF stays negative until FY2031 and the business is worth little more than its balance sheet (pro-forma net cash + investments ~HK$27/share of the ~HK$48 bear value).</t>
   </si>
   <si>
     <t xml:space="preserve">Scenario narrative: base</t>
   </si>
   <si>
-    <t xml:space="preserve">Execution risk, not impairment. Alibaba is spending the FY2026-FY2028 cash flow of the marketplace on AI compute (capex ~22% of revenue in FY2027, RMB ~250bn) and on the last leg of the quick-commerce subsidy war, so owner FCF is negative in FY2027-FY2029 and only turns in FY2030. The axes that decide the case: (1) whether AI Cloud and Compute Services keeps compounding at 30-45% with EBITA margin rising from 12% (it did in Q1 FY2027); (2) whether capex intensity actually falls after FY2028 -- the July build assumed a plateau in Y3-4, this one assumes peak absolute spend FY2027-28 and intensity normalising from FY2029; (3) whether Taobao Instant Commerce reaches unit-economics breakeven by end-FY2027 as guided while the SAMR anti-subsidy rules hold; (4) whether AI Labs/Qwen consumer losses (RMB13.9bn in one quarter) are capped rather than open-ended; (5) core CMR stays roughly flat (-7% reported / ~+1% underlying) rather than resuming share loss to PDD and Douyin. The EU DSA fine (EUR550M, booked in Q1 FY2027 G&amp;A) and the DoD 1260H litigation are carried in the discount rate, not the flows.</t>
+    <t xml:space="preserve">Execution risk, not impairment. Alibaba is spending the FY2026-FY2028 cash flow of the marketplace -- and, since 26 Aug 2026, RMB ~68bn of fresh equity -- on AI compute (capex ~23% of revenue in FY2027, RMB ~257bn) and on the last leg of the quick-commerce subsidy war, so owner FCF is negative in FY2027-FY2029 and only turns in FY2030. The axes that decide the case: (1) whether AI Cloud and Compute Services keeps compounding at 30-45% with EBITA margin rising from ~12% (Q1 FY2027: revenue +45%, EBITA +133%); (2) whether capex intensity actually falls after FY2028 -- the equity raise says the peak is being funded externally, not that it is over; (3) whether Taobao Instant Commerce reaches unit-economics breakeven by end-FY2027 as guided (Q1 showed sequential improvement at stable share) while the SAMR anti-subsidy rules hold; (4) whether AI Labs/Qwen consumer losses (RMB13.9bn in one quarter) are capped rather than open-ended; (5) core CMR stays roughly flat (-7% reported / +1% like-for-like) rather than resuming share loss to PDD and Douyin. The EU DSA fine (EUR550M, booked in Q1 FY2027 G&amp;A) and the DoD 1260H litigation are carried in the discount rate, not the flows.</t>
   </si>
   <si>
     <t xml:space="preserve">Scenario narrative: bull</t>
   </si>
   <si>
-    <t xml:space="preserve">Cloud is now a margin story as well as a growth story: 45% growth with EBITA margin doubling, Apple Intelligence embedding Qwen in the China iPhone base, Qwen3-Max-Thinking keeping Alibaba at the frontier, and the $100bn five-year external cloud+AI target on track. The same absolute capex is spread over faster revenue, so intensity normalises by FY2030; quick commerce turns profitable in FY2027 and e-commerce CMR re-accelerates on AI-driven merchant tools. Mature EBITDA margin 25%, terminal FCF margin ~12%; the 15x FCF cap binds, so the bull does not rely on a terminal multiple the market has not paid.</t>
+    <t xml:space="preserve">Cloud is now a margin story as well as a growth story: 45% growth with EBITA margin doubling, Apple Intelligence embedding Qwen in the China iPhone base, Qwen3-Max-Thinking keeping Alibaba at the frontier, AI-related product revenue (RMB12.4bn in Q1, twelfth straight triple-digit quarter) approaching a $10bn run-rate, and the $100bn five-year external cloud+AI target on track. The same absolute capex is spread over faster revenue, so intensity normalises by FY2030; quick commerce turns profitable in FY2027 and e-commerce CMR re-accelerates on AI-driven merchant tools. Mature EBITDA margin 25%, terminal FCF margin ~12%; the 15x FCF cap binds, so the bull does not rely on a terminal multiple the market has not paid.</t>
   </si>
   <si>
     <t xml:space="preserve">Item</t>
@@ -155,9 +155,6 @@
     <t xml:space="preserve">Prior valuation_date</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-07-26</t>
-  </si>
-  <si>
     <t xml:space="preserve">Prior price_then</t>
   </si>
   <si>
@@ -194,34 +191,37 @@
     <t xml:space="preserve">Bridge</t>
   </si>
   <si>
-    <t xml:space="preserve">Prior weighted IV (2026-07-26, CNYHKD 1.1597, weights 25/50/25)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Anchor refresh: CNYHKD 1.1597 -&gt; 1.1748 (+1.3%) on the prior RMB values; net cash and share count unchanged (FY2026 balance sheet is still the latest filing)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Methodology + driver change: normalised-FCF-base model replaced by component owner-FCF build with explicit capex supercycle (FY2027 capex 22% of revenue, owner FCF negative FY2027-29, recovery from FY2030), SBC and interest income stripped, single RMB-built 10% WACC (prior 11.5/10.5/13.0 was USD-rf-based), FCF-based terminal cap replacing EV/EBITDA cap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Residual after the separately-attributed items; dominated by owner FCF being negative in FY2027-29 (cum. -RMB245bn, PV -RMB210bn) where the prior model had +RMB120bn growing 22%/yr, partly offset by the lower RMB-built WACC.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bridge additions never in the prior model: strategic investments at 50% of book (+RMB224,362M)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bridge additions never in the prior model: NCI + mezzanine equity (-RMB65,384M)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weights 25/50/25 -&gt; 30/50/20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">At the prior 25/50/25 the new scenarios weight to HK$98.37.</t>
+    <t xml:space="preserve">Prior weighted IV (2026-10-22 morning build, 31 Mar 2026 balance sheet, 19,235M shares, CNYHKD 1.1748, weights 30/50/20)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anchor refresh: CNYHKD 1.1748 -&gt; 1.1750 (price move itself does not enter IV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q1 FY2027 data: balance sheet rolled to 30 Jun 2026 and share count to the Q1 diluted average</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Engine-measured total; linear decomposition at 1.175/19,324: net cash 260,828 -&gt; 207,975 (-RMB52,853M: FCF -44,670, FX -5,853, debt +6,534) -3.21; Q1 reported-FCF stub add-back +44,670 so the quarter is charged once +2.72; FY2026 dividend declared but unpaid at 30 Jun (-16,700) -1.02; shares 19,235 -&gt; 19,324 -0.43; investment portfolio 224,362 -&gt; 226,700 +0.14; NCI+mezzanine 65,384 -&gt; 64,856 +0.03. Net of the stub, the quarter's non-FCF cash leakage (FX, dividend, dilution) is what costs value.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Placing 2026-08-26: +710M shares (19,324 -&gt; 20,034M) and +RMB67,902M net proceeds (HK$79,785M at 1.175) into cash; projected capex left as is</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Issued at HK$112.70, above the weighted IV, so accretive per share overall: bear +2.32 (cash is most of the bear value), base +0.58, bull -1.25 (issued below the bull value). Equity-funding of capex already in the flows, not a reduction of that capex -- no double count.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Driver change: FY2027/FY2028 capex intensity +1pp in every scenario (base 23/21, bull 22/19, bear 24/22) on the Q1 run-rate (25% of revenue) and the compute-earmarked equity raise</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~RMB23bn of extra FY2027-28 capex in base, PV ~RMB20bn.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Driver change: SBC held at a 1.3% plateau (prior path 1.5% falling to 1.25%) on the Q1 run-rate of 1.23% and three years of declining SBC</t>
   </si>
   <si>
     <t xml:space="preserve">New weighted IV</t>
   </si>
   <si>
-    <t xml:space="preserve">ties to probability_weighted.weighted_iv</t>
+    <t xml:space="preserve">ties to probability_weighted.weighted_iv; sum of the items above = 91.50</t>
   </si>
   <si>
     <t xml:space="preserve">Period</t>
@@ -288,6 +288,18 @@
   </si>
   <si>
     <t xml:space="preserve">DividendPerShare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EBITDABeforeSignificant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RevenueContinuing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EBITDAContinuingBeforeSignificant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EBITContinuingBeforeSignificant</t>
   </si>
   <si>
     <t xml:space="preserve">Currency</t>
@@ -960,7 +972,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="0" t="n">
-        <v>103.7</v>
+        <v>101.6</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1121,52 +1133,52 @@
         <v>40</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>41</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B3" s="0" t="n">
-        <v>108.8</v>
+        <v>103.7</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B4" s="0" t="n">
-        <v>58.56</v>
+        <v>48.33</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5" s="0" t="n">
-        <v>126.99</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B6" s="0" t="n">
-        <v>182.86</v>
+        <v>149.57</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B7" s="0" t="n">
-        <v>123.85</v>
+        <v>93.31</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B8" s="0" t="s">
         <v>5</v>
@@ -1174,82 +1186,85 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B9" s="0" t="n">
-        <v>103.7</v>
+        <v>101.6</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B10" s="0" t="n">
-        <v>48.33</v>
+        <v>48.32</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B11" s="0" t="n">
-        <v>97.8</v>
+        <v>95.8</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B12" s="0" t="n">
-        <v>149.57</v>
+        <v>145.5</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B13" s="0" t="n">
-        <v>93.31</v>
+        <v>91.5</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B16" s="0" t="n">
-        <v>123.85</v>
+        <v>93.31</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B17" s="0" t="n">
-        <v>1.61</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>-1.77</v>
+      </c>
+      <c r="C18" s="0" t="s">
         <v>56</v>
-      </c>
-      <c r="B18" s="0" t="n">
-        <v>-36.8</v>
-      </c>
-      <c r="C18" s="0" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
+        <v>57</v>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="C19" s="0" t="s">
         <v>58</v>
-      </c>
-      <c r="B19" s="0" t="n">
-        <v>13.7</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1257,18 +1272,18 @@
         <v>59</v>
       </c>
       <c r="B20" s="0" t="n">
-        <v>-3.99</v>
+        <v>-1.18</v>
+      </c>
+      <c r="C20" s="0" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B21" s="0" t="n">
-        <v>-5.06</v>
-      </c>
-      <c r="C21" s="0" t="s">
-        <v>61</v>
+        <v>0.38</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1276,7 +1291,7 @@
         <v>62</v>
       </c>
       <c r="B22" s="0" t="n">
-        <v>93.31</v>
+        <v>91.5</v>
       </c>
       <c r="C22" s="0" t="s">
         <v>63</v>
@@ -1298,7 +1313,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AE11"/>
+  <dimension ref="A1:AI11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1369,19 +1384,19 @@
         <v>85</v>
       </c>
       <c r="W1" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y1" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="Z1" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="AA1" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="X1" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="Y1" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="Z1" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AA1" s="2" t="s">
-        <v>89</v>
       </c>
       <c r="AB1" s="2" t="s">
         <v>90</v>
@@ -1395,10 +1410,22 @@
       <c r="AE1" s="2" t="s">
         <v>93</v>
       </c>
+      <c r="AF1" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="AG1" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="AH1" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="AI1" s="2" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B2" s="0" t="n">
         <v>158273</v>
@@ -1445,31 +1472,31 @@
       <c r="T2" s="0" t="n">
         <v>20579</v>
       </c>
-      <c r="W2" s="0" t="s">
+      <c r="AA2" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="X2" s="0" t="s">
-        <v>95</v>
-      </c>
-      <c r="Y2" s="0" t="n">
+      <c r="AB2" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="AC2" s="0" t="n">
         <v>69172</v>
       </c>
-      <c r="Z2" s="0" t="n">
+      <c r="AD2" s="0" t="n">
         <v>127871</v>
       </c>
-      <c r="AA2" s="0" t="n">
+      <c r="AE2" s="0" t="n">
         <v>6663</v>
       </c>
-      <c r="AB2" s="0" t="n">
+      <c r="AF2" s="0" t="n">
         <v>14591</v>
       </c>
-      <c r="AC2" s="0" t="n">
+      <c r="AG2" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B3" s="0" t="n">
         <v>250266</v>
@@ -1516,25 +1543,25 @@
       <c r="T3" s="0" t="n">
         <v>20881</v>
       </c>
-      <c r="W3" s="0" t="s">
+      <c r="AA3" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="X3" s="0" t="s">
-        <v>95</v>
-      </c>
-      <c r="Y3" s="0" t="n">
+      <c r="AB3" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="AC3" s="0" t="n">
         <v>97003</v>
       </c>
-      <c r="Z3" s="0" t="n">
+      <c r="AD3" s="0" t="n">
         <v>214020</v>
       </c>
-      <c r="AA3" s="0" t="n">
+      <c r="AE3" s="0" t="n">
         <v>13390</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B4" s="0" t="n">
         <v>376844</v>
@@ -1581,31 +1608,31 @@
       <c r="T4" s="0" t="n">
         <v>20988</v>
       </c>
-      <c r="W4" s="0" t="s">
+      <c r="AA4" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="X4" s="0" t="s">
-        <v>95</v>
-      </c>
-      <c r="Y4" s="0" t="n">
+      <c r="AB4" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="AC4" s="0" t="n">
         <v>106981</v>
       </c>
-      <c r="Z4" s="0" t="n">
+      <c r="AD4" s="0" t="n">
         <v>323400</v>
       </c>
-      <c r="AA4" s="0" t="n">
+      <c r="AE4" s="0" t="n">
         <v>24702</v>
       </c>
-      <c r="AD4" s="0" t="n">
+      <c r="AH4" s="0" t="n">
         <v>3262</v>
       </c>
-      <c r="AE4" s="0" t="n">
+      <c r="AI4" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B5" s="0" t="n">
         <v>509711</v>
@@ -1652,37 +1679,37 @@
       <c r="T5" s="0" t="n">
         <v>21346</v>
       </c>
-      <c r="W5" s="0" t="s">
+      <c r="AA5" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="X5" s="0" t="s">
-        <v>95</v>
-      </c>
-      <c r="Y5" s="0" t="n">
+      <c r="AB5" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="AC5" s="0" t="n">
         <v>137136</v>
       </c>
-      <c r="Z5" s="0" t="n">
+      <c r="AD5" s="0" t="n">
         <v>379172</v>
       </c>
-      <c r="AA5" s="0" t="n">
+      <c r="AE5" s="0" t="n">
         <v>40016</v>
       </c>
-      <c r="AB5" s="0" t="n">
+      <c r="AF5" s="0" t="n">
         <v>51902</v>
       </c>
-      <c r="AC5" s="0" t="n">
+      <c r="AG5" s="0" t="n">
         <v>47286</v>
       </c>
-      <c r="AD5" s="0" t="n">
+      <c r="AH5" s="0" t="n">
         <v>28478</v>
       </c>
-      <c r="AE5" s="0" t="n">
+      <c r="AI5" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="B6" s="0" t="n">
         <v>717289</v>
@@ -1729,37 +1756,37 @@
       <c r="T6" s="0" t="n">
         <v>21982</v>
       </c>
-      <c r="W6" s="0" t="s">
+      <c r="AA6" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="X6" s="0" t="s">
-        <v>95</v>
-      </c>
-      <c r="Y6" s="0" t="n">
+      <c r="AB6" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="AC6" s="0" t="n">
         <v>170453</v>
       </c>
-      <c r="Z6" s="0" t="n">
+      <c r="AD6" s="0" t="n">
         <v>501379</v>
       </c>
-      <c r="AA6" s="0" t="n">
+      <c r="AE6" s="0" t="n">
         <v>60558</v>
       </c>
-      <c r="AB6" s="0" t="n">
+      <c r="AF6" s="0" t="n">
         <v>48851</v>
       </c>
-      <c r="AC6" s="0" t="n">
+      <c r="AG6" s="0" t="n">
         <v>37258</v>
       </c>
-      <c r="AD6" s="0" t="n">
+      <c r="AH6" s="0" t="n">
         <v>152376</v>
       </c>
-      <c r="AE6" s="0" t="n">
+      <c r="AI6" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B7" s="0" t="n">
         <v>853062</v>
@@ -1806,37 +1833,37 @@
       <c r="T7" s="0" t="n">
         <v>21787</v>
       </c>
-      <c r="W7" s="0" t="s">
+      <c r="AA7" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="X7" s="0" t="s">
-        <v>95</v>
-      </c>
-      <c r="Y7" s="0" t="n">
+      <c r="AB7" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="AC7" s="0" t="n">
         <v>130397</v>
       </c>
-      <c r="Z7" s="0" t="n">
+      <c r="AD7" s="0" t="n">
         <v>429930</v>
       </c>
-      <c r="AA7" s="0" t="n">
+      <c r="AE7" s="0" t="n">
         <v>102016</v>
       </c>
-      <c r="AB7" s="0" t="n">
+      <c r="AF7" s="0" t="n">
         <v>62185</v>
       </c>
-      <c r="AC7" s="0" t="n">
+      <c r="AG7" s="0" t="n">
         <v>66808</v>
       </c>
-      <c r="AD7" s="0" t="n">
+      <c r="AH7" s="0" t="n">
         <v>256514</v>
       </c>
-      <c r="AE7" s="0" t="n">
+      <c r="AI7" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B8" s="0" t="n">
         <v>868687</v>
@@ -1883,37 +1910,37 @@
       <c r="T8" s="0" t="n">
         <v>21114</v>
       </c>
-      <c r="W8" s="0" t="s">
+      <c r="AA8" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="X8" s="0" t="s">
-        <v>95</v>
-      </c>
-      <c r="Y8" s="0" t="n">
+      <c r="AB8" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="AC8" s="0" t="n">
         <v>147911</v>
       </c>
-      <c r="Z8" s="0" t="n">
+      <c r="AD8" s="0" t="n">
         <v>413206</v>
       </c>
-      <c r="AA8" s="0" t="n">
+      <c r="AE8" s="0" t="n">
         <v>103497</v>
       </c>
-      <c r="AB8" s="0" t="n">
+      <c r="AF8" s="0" t="n">
         <v>70506</v>
       </c>
-      <c r="AC8" s="0" t="n">
+      <c r="AG8" s="0" t="n">
         <v>77512</v>
       </c>
-      <c r="AD8" s="0" t="n">
+      <c r="AH8" s="0" t="n">
         <v>326492</v>
       </c>
-      <c r="AE8" s="0" t="n">
+      <c r="AI8" s="0" t="n">
         <v>40736</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B9" s="0" t="n">
         <v>941168</v>
@@ -1960,37 +1987,37 @@
       <c r="T9" s="0" t="n">
         <v>20359</v>
       </c>
-      <c r="W9" s="0" t="s">
+      <c r="AA9" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="X9" s="0" t="s">
-        <v>95</v>
-      </c>
-      <c r="Y9" s="0" t="n">
+      <c r="AB9" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="AC9" s="0" t="n">
         <v>165028</v>
       </c>
-      <c r="Z9" s="0" t="n">
+      <c r="AD9" s="0" t="n">
         <v>490101</v>
       </c>
-      <c r="AA9" s="0" t="n">
+      <c r="AE9" s="0" t="n">
         <v>106374</v>
       </c>
-      <c r="AB9" s="0" t="n">
+      <c r="AF9" s="0" t="n">
         <v>102598</v>
       </c>
-      <c r="AC9" s="0" t="n">
+      <c r="AG9" s="0" t="n">
         <v>99020</v>
       </c>
-      <c r="AD9" s="0" t="n">
+      <c r="AH9" s="0" t="n">
         <v>262955</v>
       </c>
-      <c r="AE9" s="0" t="n">
+      <c r="AI9" s="0" t="n">
         <v>106150</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B10" s="0" t="n">
         <v>996347</v>
@@ -2037,37 +2064,37 @@
       <c r="T10" s="0" t="n">
         <v>19318</v>
       </c>
-      <c r="W10" s="0" t="s">
+      <c r="AA10" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="X10" s="0" t="s">
-        <v>95</v>
-      </c>
-      <c r="Y10" s="0" t="n">
+      <c r="AB10" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="AC10" s="0" t="n">
         <v>173065</v>
       </c>
-      <c r="Z10" s="0" t="n">
+      <c r="AD10" s="0" t="n">
         <v>508380</v>
       </c>
-      <c r="AA10" s="0" t="n">
+      <c r="AE10" s="0" t="n">
         <v>118028</v>
       </c>
-      <c r="AB10" s="0" t="n">
+      <c r="AF10" s="0" t="n">
         <v>132300</v>
       </c>
-      <c r="AC10" s="0" t="n">
+      <c r="AG10" s="0" t="n">
         <v>101272</v>
       </c>
-      <c r="AD10" s="0" t="n">
+      <c r="AH10" s="0" t="n">
         <v>228826</v>
       </c>
-      <c r="AE10" s="0" t="n">
+      <c r="AI10" s="0" t="n">
         <v>228016</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B11" s="0" t="n">
         <v>1023670</v>
@@ -2114,31 +2141,31 @@
       <c r="T11" s="0" t="n">
         <v>19235</v>
       </c>
-      <c r="W11" s="0" t="s">
+      <c r="AA11" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="X11" s="0" t="s">
-        <v>95</v>
-      </c>
-      <c r="Y11" s="0" t="n">
+      <c r="AB11" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="AC11" s="0" t="n">
         <v>76416</v>
       </c>
-      <c r="Z11" s="0" t="n">
+      <c r="AD11" s="0" t="n">
         <v>554217</v>
       </c>
-      <c r="AA11" s="0" t="n">
+      <c r="AE11" s="0" t="n">
         <v>158132</v>
       </c>
-      <c r="AB11" s="0" t="n">
+      <c r="AF11" s="0" t="n">
         <v>144170</v>
       </c>
-      <c r="AC11" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD11" s="0" t="n">
+      <c r="AG11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH11" s="0" t="n">
         <v>155310</v>
       </c>
-      <c r="AE11" s="0" t="n">
+      <c r="AI11" s="0" t="n">
         <v>238075</v>
       </c>
     </row>
@@ -2166,7 +2193,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>38</v>
@@ -2174,39 +2201,39 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>103.7</v>
+        <v>101.6</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>19235</v>
+        <v>20034</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>-260828</v>
+        <v>-275877</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>158978</v>
+        <v>189814</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B6" s="3" t="n">
         <v>15</v>
@@ -2214,7 +2241,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B7" s="3" t="n">
         <v>1023670</v>
@@ -2222,66 +2249,66 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="B10" s="3" t="n">
-        <v>1.1748</v>
+        <v>1.175</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C13" s="3" t="n">
         <v>6</v>
@@ -2316,7 +2343,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C14" s="3" t="n">
         <v>12</v>
@@ -2351,25 +2378,25 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>1.45</v>
+        <v>1.3</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>1.35</v>
+        <v>1.3</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>1.3</v>
@@ -2386,7 +2413,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C16" s="3" t="n">
         <v>0</v>
@@ -2421,7 +2448,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C17" s="3" t="n">
         <v>5.5</v>
@@ -2456,13 +2483,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>17</v>
@@ -2491,7 +2518,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C19" s="3" t="n">
         <v>18</v>
@@ -2526,7 +2553,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B20" s="3" t="n">
         <v>10</v>
@@ -2534,7 +2561,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B21" s="3" t="n">
         <v>2</v>
@@ -2542,7 +2569,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B22" s="3" t="n">
         <v>12</v>
@@ -2550,7 +2577,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B23" s="3" t="n">
         <v>0</v>
@@ -2558,7 +2585,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B24" s="3" t="n">
         <v>0.3</v>
@@ -2566,42 +2593,42 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C27" s="3" t="n">
         <v>9</v>
@@ -2636,7 +2663,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C28" s="3" t="n">
         <v>13.5</v>
@@ -2671,25 +2698,25 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C29" s="3" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>1.45</v>
+        <v>1.3</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>1.35</v>
+        <v>1.3</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>1.3</v>
@@ -2706,7 +2733,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C30" s="3" t="n">
         <v>0</v>
@@ -2741,7 +2768,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C31" s="3" t="n">
         <v>5.5</v>
@@ -2776,13 +2803,13 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="C32" s="3" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E32" s="3" t="n">
         <v>17</v>
@@ -2811,7 +2838,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C33" s="3" t="n">
         <v>18</v>
@@ -2846,7 +2873,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B34" s="3" t="n">
         <v>10</v>
@@ -2854,7 +2881,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B35" s="3" t="n">
         <v>3</v>
@@ -2862,7 +2889,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B36" s="3" t="n">
         <v>15</v>
@@ -2870,7 +2897,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B37" s="3" t="n">
         <v>0</v>
@@ -2878,7 +2905,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B38" s="3" t="n">
         <v>0.5</v>
@@ -2886,42 +2913,42 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="L40" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C41" s="3" t="n">
         <v>11</v>
@@ -2956,7 +2983,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C42" s="3" t="n">
         <v>14.5</v>
@@ -2991,25 +3018,25 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C43" s="3" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>1.45</v>
+        <v>1.3</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>1.35</v>
+        <v>1.3</v>
       </c>
       <c r="I43" s="3" t="n">
         <v>1.3</v>
@@ -3026,7 +3053,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C44" s="3" t="n">
         <v>0</v>
@@ -3061,7 +3088,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C45" s="3" t="n">
         <v>5.5</v>
@@ -3096,13 +3123,13 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="0" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="C46" s="3" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E46" s="3" t="n">
         <v>15</v>
@@ -3131,7 +3158,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C47" s="3" t="n">
         <v>18</v>
@@ -3166,7 +3193,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B48" s="3" t="n">
         <v>10</v>
@@ -3174,7 +3201,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B49" s="3" t="n">
         <v>3.5</v>
@@ -3182,7 +3209,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B50" s="3" t="n">
         <v>15</v>
@@ -3190,7 +3217,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B51" s="3" t="n">
         <v>0</v>
@@ -3198,7 +3225,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B52" s="3" t="n">
         <v>0.2</v>
@@ -3228,50 +3255,50 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B4" s="0" t="n">
         <v>0</v>
@@ -3319,7 +3346,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C5" s="4" t="n">
         <f aca="false">Assumptions!C13</f>
@@ -3412,7 +3439,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C7" s="4" t="n">
         <f aca="false">Assumptions!C14</f>
@@ -3502,31 +3529,31 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C9" s="4" t="n">
         <f aca="false">Assumptions!C15</f>
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="D9" s="4" t="n">
         <f aca="false">Assumptions!D15</f>
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="E9" s="4" t="n">
         <f aca="false">Assumptions!E15</f>
-        <v>1.45</v>
+        <v>1.3</v>
       </c>
       <c r="F9" s="4" t="n">
         <f aca="false">Assumptions!F15</f>
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="G9" s="4" t="n">
         <f aca="false">Assumptions!G15</f>
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="H9" s="4" t="n">
         <f aca="false">Assumptions!H15</f>
-        <v>1.35</v>
+        <v>1.3</v>
       </c>
       <c r="I9" s="4" t="n">
         <f aca="false">Assumptions!I15</f>
@@ -3547,31 +3574,31 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C10" s="0" t="n">
         <f aca="false">-C6*C9/100</f>
-        <v>-16276.353</v>
+        <v>-14106.1726</v>
       </c>
       <c r="D10" s="0" t="n">
         <f aca="false">-D6*D9/100</f>
-        <v>-17090.17065</v>
+        <v>-14811.48123</v>
       </c>
       <c r="E10" s="0" t="n">
         <f aca="false">-E6*E9/100</f>
-        <v>-17263.920718275</v>
+        <v>-15477.99788535</v>
       </c>
       <c r="F10" s="0" t="n">
         <f aca="false">-F6*F9/100</f>
-        <v>-17335.357631592</v>
+        <v>-16097.117800764</v>
       </c>
       <c r="G10" s="0" t="n">
         <f aca="false">-G6*G9/100</f>
-        <v>-17942.0951486977</v>
+        <v>-16660.5169237907</v>
       </c>
       <c r="H10" s="0" t="n">
         <f aca="false">-H6*H9/100</f>
-        <v>-17820.3452173316</v>
+        <v>-17160.3324315045</v>
       </c>
       <c r="I10" s="0" t="n">
         <f aca="false">-I6*I9/100</f>
@@ -3592,31 +3619,31 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="C11" s="0" t="n">
         <f aca="false">C8+C10+C24</f>
-        <v>113934.471</v>
+        <v>116104.6514</v>
       </c>
       <c r="D11" s="0" t="n">
         <f aca="false">D8+D10+D24</f>
-        <v>131024.64165</v>
+        <v>133303.33107</v>
       </c>
       <c r="E11" s="0" t="n">
         <f aca="false">E8+E10+E24</f>
-        <v>149422.210354725</v>
+        <v>151208.13318765</v>
       </c>
       <c r="F11" s="0" t="n">
         <f aca="false">F8+F10+F24</f>
-        <v>168400.616992608</v>
+        <v>169638.856823436</v>
       </c>
       <c r="G11" s="0" t="n">
         <f aca="false">G8+G10+G24</f>
-        <v>180702.529711884</v>
+        <v>181984.107936791</v>
       </c>
       <c r="H11" s="0" t="n">
         <f aca="false">H8+H10+H24</f>
-        <v>193383.746247339</v>
+        <v>194043.759033166</v>
       </c>
       <c r="I11" s="0" t="n">
         <f aca="false">I8+I10+I24</f>
@@ -3637,7 +3664,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="C12" s="4" t="n">
         <f aca="false">-C6*Assumptions!C17/100</f>
@@ -3682,31 +3709,31 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C13" s="0" t="n">
         <f aca="false">C11+C12</f>
-        <v>54254.51</v>
+        <v>56424.6904</v>
       </c>
       <c r="D13" s="0" t="n">
         <f aca="false">D11+D12</f>
-        <v>45573.7884</v>
+        <v>47852.47782</v>
       </c>
       <c r="E13" s="0" t="n">
         <f aca="false">E11+E12</f>
-        <v>36313.764269475</v>
+        <v>38099.6871024</v>
       </c>
       <c r="F13" s="0" t="n">
         <f aca="false">F11+F12</f>
-        <v>38385.434755668</v>
+        <v>39623.674586496</v>
       </c>
       <c r="G13" s="0" t="n">
         <f aca="false">G11+G12</f>
-        <v>46136.8160966513</v>
+        <v>47418.3943215582</v>
       </c>
       <c r="H13" s="0" t="n">
         <f aca="false">H11+H12</f>
-        <v>61381.1890819198</v>
+        <v>62041.2018677469</v>
       </c>
       <c r="I13" s="0" t="n">
         <f aca="false">I11+I12</f>
@@ -3727,7 +3754,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C14" s="4" t="n">
         <f aca="false">Assumptions!C19</f>
@@ -3772,31 +3799,31 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C15" s="0" t="n">
         <f aca="false">C13-MAX(0,C13)*C14/100</f>
-        <v>44488.6982</v>
+        <v>46268.246128</v>
       </c>
       <c r="D15" s="0" t="n">
         <f aca="false">D13-MAX(0,D13)*D14/100</f>
-        <v>37370.506488</v>
+        <v>39239.0318124</v>
       </c>
       <c r="E15" s="0" t="n">
         <f aca="false">E13-MAX(0,E13)*E14/100</f>
-        <v>29777.2867009695</v>
+        <v>31241.743423968</v>
       </c>
       <c r="F15" s="0" t="n">
         <f aca="false">F13-MAX(0,F13)*F14/100</f>
-        <v>31476.0564996477</v>
+        <v>32491.4131609267</v>
       </c>
       <c r="G15" s="0" t="n">
         <f aca="false">G13-MAX(0,G13)*G14/100</f>
-        <v>37832.189199254</v>
+        <v>38883.0833436778</v>
       </c>
       <c r="H15" s="0" t="n">
         <f aca="false">H13-MAX(0,H13)*H14/100</f>
-        <v>50332.5750471742</v>
+        <v>50873.7855315525</v>
       </c>
       <c r="I15" s="0" t="n">
         <f aca="false">I13-MAX(0,I13)*I14/100</f>
@@ -3817,7 +3844,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="C16" s="0" t="n">
         <f aca="false">-C12</f>
@@ -3862,15 +3889,15 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C17" s="4" t="n">
         <f aca="false">-C6*Assumptions!C18/100</f>
-        <v>-249570.746</v>
+        <v>-260421.648</v>
       </c>
       <c r="D17" s="4" t="n">
         <f aca="false">-D6*Assumptions!D18/100</f>
-        <v>-239262.3891</v>
+        <v>-250655.8362</v>
       </c>
       <c r="E17" s="4" t="n">
         <f aca="false">-E6*Assumptions!E18/100</f>
@@ -3907,7 +3934,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="C18" s="4" t="n">
         <f aca="false">(C6-B6)*Assumptions!$B$23/100</f>
@@ -3952,31 +3979,31 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C19" s="0" t="n">
         <f aca="false">C15+C16+C17+C18</f>
-        <v>-145402.0868</v>
+        <v>-154473.440872</v>
       </c>
       <c r="D19" s="0" t="n">
         <f aca="false">D15+D16+D17+D18</f>
-        <v>-116441.029362</v>
+        <v>-125965.9511376</v>
       </c>
       <c r="E19" s="0" t="n">
         <f aca="false">E15+E16+E17+E18</f>
-        <v>-59518.8549452805</v>
+        <v>-58054.398222282</v>
       </c>
       <c r="F19" s="0" t="n">
         <f aca="false">F15+F16+F17+F18</f>
-        <v>520.060728947778</v>
+        <v>1535.41739022671</v>
       </c>
       <c r="G19" s="0" t="n">
         <f aca="false">G15+G16+G17+G18</f>
-        <v>37832.189199254</v>
+        <v>38883.0833436778</v>
       </c>
       <c r="H19" s="0" t="n">
         <f aca="false">H15+H16+H17+H18</f>
-        <v>63532.8307637161</v>
+        <v>64074.0412480944</v>
       </c>
       <c r="I19" s="0" t="n">
         <f aca="false">I15+I16+I17+I18</f>
@@ -3997,7 +4024,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="C20" s="0" t="n">
         <f aca="false">1/(1+$B$27/100)^C4</f>
@@ -4042,31 +4069,31 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="C21" s="0" t="n">
         <f aca="false">C19*C20</f>
-        <v>-132183.715272727</v>
+        <v>-140430.400792727</v>
       </c>
       <c r="D21" s="0" t="n">
         <f aca="false">D19*D20</f>
-        <v>-96232.2556710744</v>
+        <v>-104104.091849256</v>
       </c>
       <c r="E21" s="0" t="n">
         <f aca="false">E19*E20</f>
-        <v>-44717.3966531033</v>
+        <v>-43617.1286418347</v>
       </c>
       <c r="F21" s="0" t="n">
         <f aca="false">F19*F20</f>
-        <v>355.208475478299</v>
+        <v>1048.71073712636</v>
       </c>
       <c r="G21" s="0" t="n">
         <f aca="false">G19*G20</f>
-        <v>23490.8129718251</v>
+        <v>24143.3355543758</v>
       </c>
       <c r="H21" s="0" t="n">
         <f aca="false">H19*H20</f>
-        <v>35862.6266686364</v>
+        <v>36168.1258777396</v>
       </c>
       <c r="I21" s="0" t="n">
         <f aca="false">I19*I20</f>
@@ -4087,7 +4114,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C23" s="4" t="n">
         <f aca="false">Assumptions!C16</f>
@@ -4132,7 +4159,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C24" s="0" t="n">
         <f aca="false">-C6*C23/100</f>
@@ -4177,12 +4204,12 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B27" s="4" t="n">
         <f aca="false">Assumptions!$B$20</f>
@@ -4191,7 +4218,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B28" s="4" t="n">
         <f aca="false">Assumptions!$B$21</f>
@@ -4200,7 +4227,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B29" s="4" t="n">
         <f aca="false">Assumptions!$B$22</f>
@@ -4209,16 +4236,16 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="B30" s="0" t="n">
         <f aca="false">SUM(C21:L21)</f>
-        <v>-56874.2549860303</v>
+        <v>-70240.9846196415</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="B31" s="0" t="n">
         <f aca="false">L19</f>
@@ -4227,7 +4254,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="B32" s="0" t="n">
         <f aca="false">IF(B27&gt;B28,B31*(1+B28/100)/((B27-B28)/100),B31*B29)</f>
@@ -4236,7 +4263,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B33" s="0" t="n">
         <f aca="false">B31*B29</f>
@@ -4245,7 +4272,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="B34" s="0" t="n">
         <f aca="false">MAX(0,MIN(B32,B33))</f>
@@ -4254,7 +4281,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B35" s="0" t="n">
         <f aca="false">B34/(1+B27/100)^L4</f>
@@ -4263,52 +4290,52 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="B36" s="0" t="n">
         <f aca="false">B30+B35</f>
-        <v>371513.867532022</v>
+        <v>358147.13789841</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="B37" s="0" t="n">
         <f aca="false">B36+Assumptions!$B$5-Assumptions!$B$4</f>
-        <v>791319.867532022</v>
+        <v>823838.13789841</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="B38" s="0" t="n">
         <f aca="false">B37/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>48.3307814076745</v>
+        <v>48.3183494075388</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="B39" s="4" t="n">
         <f aca="false">B38/Assumptions!$B$2-1</f>
-        <v>-0.533936534159359</v>
+        <v>-0.524425694807689</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B41" s="0" t="n">
         <f aca="false">SUMPRODUCT(-C10:L10/(1+$B$27/100)^C4:L4)</f>
-        <v>107047.733349101</v>
+        <v>99835.783698496</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="B42" s="0" t="n">
         <f aca="false">IF(B27&gt;B28,-L10*(1+B28/100)/((B27-B28)/100),-L10*20)/(1+B27/100)^L4</f>
@@ -4317,16 +4344,16 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B43" s="0" t="n">
         <f aca="false">(B37+B41+B42)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>60.3368973528279</v>
+        <v>59.4246144865056</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B45" s="4" t="n">
         <f aca="false">Assumptions!$B$6</f>
@@ -4335,7 +4362,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="0" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="B46" s="0" t="n">
         <f aca="false">MAX(0,MIN(IF(B45&gt;B28,B31*(1+B28/100)/((B45-B28)/100),B31*B29),B31*B29))</f>
@@ -4344,11 +4371,11 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="B47" s="0" t="n">
         <f aca="false">(SUMPRODUCT(C19:L19/(1+B45/100)^C4:L4)+B46/(1+B45/100)^L4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>30.5373932118357</v>
+        <v>31.2654915572399</v>
       </c>
     </row>
   </sheetData>
@@ -4375,50 +4402,50 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B4" s="0" t="n">
         <v>0</v>
@@ -4466,7 +4493,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C5" s="4" t="n">
         <f aca="false">Assumptions!C27</f>
@@ -4559,7 +4586,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C7" s="4" t="n">
         <f aca="false">Assumptions!C28</f>
@@ -4649,31 +4676,31 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C9" s="4" t="n">
         <f aca="false">Assumptions!C29</f>
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="D9" s="4" t="n">
         <f aca="false">Assumptions!D29</f>
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="E9" s="4" t="n">
         <f aca="false">Assumptions!E29</f>
-        <v>1.45</v>
+        <v>1.3</v>
       </c>
       <c r="F9" s="4" t="n">
         <f aca="false">Assumptions!F29</f>
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="G9" s="4" t="n">
         <f aca="false">Assumptions!G29</f>
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="H9" s="4" t="n">
         <f aca="false">Assumptions!H29</f>
-        <v>1.35</v>
+        <v>1.3</v>
       </c>
       <c r="I9" s="4" t="n">
         <f aca="false">Assumptions!I29</f>
@@ -4694,31 +4721,31 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C10" s="0" t="n">
         <f aca="false">-C6*C9/100</f>
-        <v>-16737.0045</v>
+        <v>-14505.4039</v>
       </c>
       <c r="D10" s="0" t="n">
         <f aca="false">-D6*D9/100</f>
-        <v>-18243.334905</v>
+        <v>-15810.890251</v>
       </c>
       <c r="E10" s="0" t="n">
         <f aca="false">-E6*E9/100</f>
-        <v>-19134.2177595275</v>
+        <v>-17154.815922335</v>
       </c>
       <c r="F10" s="0" t="n">
         <f aca="false">-F6*F9/100</f>
-        <v>-19952.3705189004</v>
+        <v>-18527.2011961218</v>
       </c>
       <c r="G10" s="0" t="n">
         <f aca="false">-G6*G9/100</f>
-        <v>-21349.0364552234</v>
+        <v>-19824.1052798503</v>
       </c>
       <c r="H10" s="0" t="n">
         <f aca="false">-H6*H9/100</f>
-        <v>-21821.7651195891</v>
+        <v>-21013.5515966414</v>
       </c>
       <c r="I10" s="0" t="n">
         <f aca="false">-I6*I9/100</f>
@@ -4739,31 +4766,31 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="C11" s="0" t="n">
         <f aca="false">C8+C10+C24</f>
-        <v>133896.036</v>
+        <v>136127.6366</v>
       </c>
       <c r="D11" s="0" t="n">
         <f aca="false">D8+D10+D24</f>
-        <v>170271.12578</v>
+        <v>172703.570434</v>
       </c>
       <c r="E11" s="0" t="n">
         <f aca="false">E8+E10+E24</f>
-        <v>205197.990455622</v>
+        <v>207177.392292815</v>
       </c>
       <c r="F11" s="0" t="n">
         <f aca="false">F8+F10+F24</f>
-        <v>243703.954195141</v>
+        <v>245129.123517919</v>
       </c>
       <c r="G11" s="0" t="n">
         <f aca="false">G8+G10+G24</f>
-        <v>276012.542742531</v>
+        <v>277537.473917905</v>
       </c>
       <c r="H11" s="0" t="n">
         <f aca="false">H8+H10+H24</f>
-        <v>309545.779288986</v>
+        <v>310353.992811934</v>
       </c>
       <c r="I11" s="0" t="n">
         <f aca="false">I8+I10+I24</f>
@@ -4784,7 +4811,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="C12" s="4" t="n">
         <f aca="false">-C6*Assumptions!C31/100</f>
@@ -4829,31 +4856,31 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C13" s="0" t="n">
         <f aca="false">C11+C12</f>
-        <v>72527.0195</v>
+        <v>74758.6201</v>
       </c>
       <c r="D13" s="0" t="n">
         <f aca="false">D11+D12</f>
-        <v>79054.451255</v>
+        <v>81486.895909</v>
       </c>
       <c r="E13" s="0" t="n">
         <f aca="false">E11+E12</f>
-        <v>86433.8802240725</v>
+        <v>88413.282061265</v>
       </c>
       <c r="F13" s="0" t="n">
         <f aca="false">F11+F12</f>
-        <v>101187.021917281</v>
+        <v>102612.191240059</v>
       </c>
       <c r="G13" s="0" t="n">
         <f aca="false">G11+G12</f>
-        <v>123519.425205221</v>
+        <v>125044.356380594</v>
       </c>
       <c r="H13" s="0" t="n">
         <f aca="false">H11+H12</f>
-        <v>155985.209928915</v>
+        <v>156793.423451862</v>
       </c>
       <c r="I13" s="0" t="n">
         <f aca="false">I11+I12</f>
@@ -4874,7 +4901,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C14" s="4" t="n">
         <f aca="false">Assumptions!C33</f>
@@ -4919,31 +4946,31 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C15" s="0" t="n">
         <f aca="false">C13-MAX(0,C13)*C14/100</f>
-        <v>59472.15599</v>
+        <v>61302.068482</v>
       </c>
       <c r="D15" s="0" t="n">
         <f aca="false">D13-MAX(0,D13)*D14/100</f>
-        <v>64824.6500291</v>
+        <v>66819.25464538</v>
       </c>
       <c r="E15" s="0" t="n">
         <f aca="false">E13-MAX(0,E13)*E14/100</f>
-        <v>70875.7817837394</v>
+        <v>72498.8912902373</v>
       </c>
       <c r="F15" s="0" t="n">
         <f aca="false">F13-MAX(0,F13)*F14/100</f>
-        <v>82973.3579721701</v>
+        <v>84141.9968168486</v>
       </c>
       <c r="G15" s="0" t="n">
         <f aca="false">G13-MAX(0,G13)*G14/100</f>
-        <v>101285.928668281</v>
+        <v>102536.372232087</v>
       </c>
       <c r="H15" s="0" t="n">
         <f aca="false">H13-MAX(0,H13)*H14/100</f>
-        <v>127907.87214171</v>
+        <v>128570.607230527</v>
       </c>
       <c r="I15" s="0" t="n">
         <f aca="false">I13-MAX(0,I13)*I14/100</f>
@@ -4964,7 +4991,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="C16" s="0" t="n">
         <f aca="false">-C12</f>
@@ -5009,15 +5036,15 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C17" s="4" t="n">
         <f aca="false">-C6*Assumptions!C32/100</f>
-        <v>-245476.066</v>
+        <v>-256634.069</v>
       </c>
       <c r="D17" s="4" t="n">
         <f aca="false">-D6*Assumptions!D32/100</f>
-        <v>-243244.4654</v>
+        <v>-255406.68867</v>
       </c>
       <c r="E17" s="4" t="n">
         <f aca="false">-E6*Assumptions!E32/100</f>
@@ -5054,7 +5081,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="C18" s="4" t="n">
         <f aca="false">(C6-B6)*Assumptions!$B$37/100</f>
@@ -5099,31 +5126,31 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C19" s="0" t="n">
         <f aca="false">C15+C16+C17+C18</f>
-        <v>-124634.89351</v>
+        <v>-133962.984018</v>
       </c>
       <c r="D19" s="0" t="n">
         <f aca="false">D15+D16+D17+D18</f>
-        <v>-87203.1408459</v>
+        <v>-97370.75949962</v>
       </c>
       <c r="E19" s="0" t="n">
         <f aca="false">E15+E16+E17+E18</f>
-        <v>-34692.3161998605</v>
+        <v>-33069.2066933627</v>
       </c>
       <c r="F19" s="0" t="n">
         <f aca="false">F15+F16+F17+F18</f>
-        <v>18840.7384471331</v>
+        <v>20009.3772918115</v>
       </c>
       <c r="G19" s="0" t="n">
         <f aca="false">G15+G16+G17+G18</f>
-        <v>63162.6492839539</v>
+        <v>64413.0928477598</v>
       </c>
       <c r="H19" s="0" t="n">
         <f aca="false">H15+H16+H17+H18</f>
-        <v>103661.466453278</v>
+        <v>104324.201542095</v>
       </c>
       <c r="I19" s="0" t="n">
         <f aca="false">I15+I16+I17+I18</f>
@@ -5144,7 +5171,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="C20" s="0" t="n">
         <f aca="false">1/(1+$B$27/100)^C4</f>
@@ -5189,31 +5216,31 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="C21" s="0" t="n">
         <f aca="false">C19*C20</f>
-        <v>-113304.448645455</v>
+        <v>-121784.530925455</v>
       </c>
       <c r="D21" s="0" t="n">
         <f aca="false">D19*D20</f>
-        <v>-72068.7114428926</v>
+        <v>-80471.7020658017</v>
       </c>
       <c r="E21" s="0" t="n">
         <f aca="false">E19*E20</f>
-        <v>-26064.8506385128</v>
+        <v>-24845.3844427969</v>
       </c>
       <c r="F21" s="0" t="n">
         <f aca="false">F19*F20</f>
-        <v>12868.4778684059</v>
+        <v>13666.6739237836</v>
       </c>
       <c r="G21" s="0" t="n">
         <f aca="false">G19*G20</f>
-        <v>39219.035761314</v>
+        <v>39995.4628333632</v>
       </c>
       <c r="H21" s="0" t="n">
         <f aca="false">H19*H20</f>
-        <v>58514.1953640194</v>
+        <v>58888.2920441886</v>
       </c>
       <c r="I21" s="0" t="n">
         <f aca="false">I19*I20</f>
@@ -5234,7 +5261,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C23" s="4" t="n">
         <f aca="false">Assumptions!C30</f>
@@ -5279,7 +5306,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C24" s="0" t="n">
         <f aca="false">-C6*C23/100</f>
@@ -5324,12 +5351,12 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B27" s="4" t="n">
         <f aca="false">Assumptions!$B$34</f>
@@ -5338,7 +5365,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B28" s="4" t="n">
         <f aca="false">Assumptions!$B$35</f>
@@ -5347,7 +5374,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B29" s="4" t="n">
         <f aca="false">Assumptions!$B$36</f>
@@ -5356,16 +5383,16 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="B30" s="0" t="n">
         <f aca="false">SUM(C21:L21)</f>
-        <v>172998.903954538</v>
+        <v>159284.017054941</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="B31" s="0" t="n">
         <f aca="false">L19</f>
@@ -5374,7 +5401,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="B32" s="0" t="n">
         <f aca="false">IF(B27&gt;B28,B31*(1+B28/100)/((B27-B28)/100),B31*B29)</f>
@@ -5383,7 +5410,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B33" s="0" t="n">
         <f aca="false">B31*B29</f>
@@ -5392,7 +5419,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="B34" s="0" t="n">
         <f aca="false">MAX(0,MIN(B32,B33))</f>
@@ -5401,7 +5428,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B35" s="0" t="n">
         <f aca="false">B34/(1+B27/100)^L4</f>
@@ -5410,52 +5437,52 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="B36" s="0" t="n">
         <f aca="false">B30+B35</f>
-        <v>1181481.4393973</v>
+        <v>1167766.55249771</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="B37" s="0" t="n">
         <f aca="false">B36+Assumptions!$B$5-Assumptions!$B$4</f>
-        <v>1601287.4393973</v>
+        <v>1633457.55249771</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="B38" s="0" t="n">
         <f aca="false">B37/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>97.8004930493348</v>
+        <v>95.8027665061798</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="B39" s="4" t="n">
         <f aca="false">B38/Assumptions!$B$2-1</f>
-        <v>-0.0568901345290768</v>
+        <v>-0.0570593847816948</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B41" s="0" t="n">
         <f aca="false">SUMPRODUCT(-C10:L10/(1+$B$27/100)^C4:L4)</f>
-        <v>125403.59154643</v>
+        <v>117500.937422778</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="B42" s="0" t="n">
         <f aca="false">IF(B27&gt;B28,-L10*(1+B28/100)/((B27-B28)/100),-L10*20)/(1+B27/100)^L4</f>
@@ -5464,16 +5491,16 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B43" s="0" t="n">
         <f aca="false">(B37+B41+B42)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>113.887994416978</v>
+        <v>110.787799467257</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B45" s="4" t="n">
         <f aca="false">Assumptions!$B$6</f>
@@ -5482,7 +5509,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="0" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="B46" s="0" t="n">
         <f aca="false">MAX(0,MIN(IF(B45&gt;B28,B31*(1+B28/100)/((B45-B28)/100),B31*B29),B31*B29))</f>
@@ -5491,11 +5518,11 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="B47" s="0" t="n">
         <f aca="false">(SUMPRODUCT(C19:L19/(1+B45/100)^C4:L4)+B46/(1+B45/100)^L4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>53.410096657993</v>
+        <v>53.2082823457069</v>
       </c>
     </row>
   </sheetData>
@@ -5522,50 +5549,50 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B4" s="0" t="n">
         <v>0</v>
@@ -5613,7 +5640,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C5" s="4" t="n">
         <f aca="false">Assumptions!C41</f>
@@ -5706,7 +5733,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C7" s="4" t="n">
         <f aca="false">Assumptions!C42</f>
@@ -5796,31 +5823,31 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C9" s="4" t="n">
         <f aca="false">Assumptions!C43</f>
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="D9" s="4" t="n">
         <f aca="false">Assumptions!D43</f>
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="E9" s="4" t="n">
         <f aca="false">Assumptions!E43</f>
-        <v>1.45</v>
+        <v>1.3</v>
       </c>
       <c r="F9" s="4" t="n">
         <f aca="false">Assumptions!F43</f>
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="G9" s="4" t="n">
         <f aca="false">Assumptions!G43</f>
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="H9" s="4" t="n">
         <f aca="false">Assumptions!H43</f>
-        <v>1.35</v>
+        <v>1.3</v>
       </c>
       <c r="I9" s="4" t="n">
         <f aca="false">Assumptions!I43</f>
@@ -5841,31 +5868,31 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C10" s="0" t="n">
         <f aca="false">-C6*C9/100</f>
-        <v>-17044.1055</v>
+        <v>-14771.5581</v>
       </c>
       <c r="D10" s="0" t="n">
         <f aca="false">-D6*D9/100</f>
-        <v>-18918.957105</v>
+        <v>-16396.429491</v>
       </c>
       <c r="E10" s="0" t="n">
         <f aca="false">-E6*E9/100</f>
-        <v>-20117.15772165</v>
+        <v>-18036.0724401</v>
       </c>
       <c r="F10" s="0" t="n">
         <f aca="false">-F6*F9/100</f>
-        <v>-21171.574264302</v>
+        <v>-19659.318959709</v>
       </c>
       <c r="G10" s="0" t="n">
         <f aca="false">-G6*G9/100</f>
-        <v>-22865.3002054462</v>
+        <v>-21232.0644764857</v>
       </c>
       <c r="H10" s="0" t="n">
         <f aca="false">-H6*H9/100</f>
-        <v>-23592.0901048336</v>
+        <v>-22718.3089898397</v>
       </c>
       <c r="I10" s="0" t="n">
         <f aca="false">-I6*I9/100</f>
@@ -5886,31 +5913,31 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="C11" s="0" t="n">
         <f aca="false">C8+C10+C24</f>
-        <v>147715.581</v>
+        <v>149988.1284</v>
       </c>
       <c r="D11" s="0" t="n">
         <f aca="false">D8+D10+D24</f>
-        <v>201802.20912</v>
+        <v>204324.736734</v>
       </c>
       <c r="E11" s="0" t="n">
         <f aca="false">E8+E10+E24</f>
-        <v>250423.92887985</v>
+        <v>252505.0141614</v>
       </c>
       <c r="F11" s="0" t="n">
         <f aca="false">F8+F10+F24</f>
-        <v>303963.316223193</v>
+        <v>305475.571527786</v>
       </c>
       <c r="G11" s="0" t="n">
         <f aca="false">G8+G10+G24</f>
-        <v>352778.917455455</v>
+        <v>354412.153184416</v>
       </c>
       <c r="H11" s="0" t="n">
         <f aca="false">H8+H10+H24</f>
-        <v>395822.845092208</v>
+        <v>396696.626207201</v>
       </c>
       <c r="I11" s="0" t="n">
         <f aca="false">I8+I10+I24</f>
@@ -5931,7 +5958,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="C12" s="4" t="n">
         <f aca="false">-C6*Assumptions!C45/100</f>
@@ -5976,31 +6003,31 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C13" s="0" t="n">
         <f aca="false">C11+C12</f>
-        <v>85220.5275</v>
+        <v>87493.0749</v>
       </c>
       <c r="D13" s="0" t="n">
         <f aca="false">D11+D12</f>
-        <v>113513.74263</v>
+        <v>116036.270244</v>
       </c>
       <c r="E13" s="0" t="n">
         <f aca="false">E11+E12</f>
-        <v>132495.76292535</v>
+        <v>134576.8482069</v>
       </c>
       <c r="F13" s="0" t="n">
         <f aca="false">F11+F12</f>
-        <v>167860.338809823</v>
+        <v>169372.594114416</v>
       </c>
       <c r="G13" s="0" t="n">
         <f aca="false">G11+G12</f>
-        <v>205787.701849016</v>
+        <v>207420.937577976</v>
       </c>
       <c r="H13" s="0" t="n">
         <f aca="false">H11+H12</f>
-        <v>238542.244393317</v>
+        <v>239416.025508311</v>
       </c>
       <c r="I13" s="0" t="n">
         <f aca="false">I11+I12</f>
@@ -6021,7 +6048,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C14" s="4" t="n">
         <f aca="false">Assumptions!C47</f>
@@ -6066,31 +6093,31 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C15" s="0" t="n">
         <f aca="false">C13-MAX(0,C13)*C14/100</f>
-        <v>69880.83255</v>
+        <v>71744.321418</v>
       </c>
       <c r="D15" s="0" t="n">
         <f aca="false">D13-MAX(0,D13)*D14/100</f>
-        <v>93081.2689566</v>
+        <v>95149.74160008</v>
       </c>
       <c r="E15" s="0" t="n">
         <f aca="false">E13-MAX(0,E13)*E14/100</f>
-        <v>108646.525598787</v>
+        <v>110353.015529658</v>
       </c>
       <c r="F15" s="0" t="n">
         <f aca="false">F13-MAX(0,F13)*F14/100</f>
-        <v>137645.477824055</v>
+        <v>138885.527173821</v>
       </c>
       <c r="G15" s="0" t="n">
         <f aca="false">G13-MAX(0,G13)*G14/100</f>
-        <v>168745.915516193</v>
+        <v>170085.16881394</v>
       </c>
       <c r="H15" s="0" t="n">
         <f aca="false">H13-MAX(0,H13)*H14/100</f>
-        <v>195604.64040252</v>
+        <v>196321.140916815</v>
       </c>
       <c r="I15" s="0" t="n">
         <f aca="false">I13-MAX(0,I13)*I14/100</f>
@@ -6111,7 +6138,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="C16" s="0" t="n">
         <f aca="false">-C12</f>
@@ -6156,15 +6183,15 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C17" s="4" t="n">
         <f aca="false">-C6*Assumptions!C46/100</f>
-        <v>-238617.477</v>
+        <v>-249980.214</v>
       </c>
       <c r="D17" s="4" t="n">
         <f aca="false">-D6*Assumptions!D46/100</f>
-        <v>-227027.48526</v>
+        <v>-239640.12333</v>
       </c>
       <c r="E17" s="4" t="n">
         <f aca="false">-E6*Assumptions!E46/100</f>
@@ -6201,7 +6228,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="C18" s="4" t="n">
         <f aca="false">(C6-B6)*Assumptions!$B$51/100</f>
@@ -6246,31 +6273,31 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C19" s="0" t="n">
         <f aca="false">C15+C16+C17+C18</f>
-        <v>-106241.59095</v>
+        <v>-115740.839082</v>
       </c>
       <c r="D19" s="0" t="n">
         <f aca="false">D15+D16+D17+D18</f>
-        <v>-45657.7498134</v>
+        <v>-56201.91523992</v>
       </c>
       <c r="E19" s="0" t="n">
         <f aca="false">E15+E16+E17+E18</f>
-        <v>18466.163398287</v>
+        <v>20172.653329158</v>
       </c>
       <c r="F19" s="0" t="n">
         <f aca="false">F15+F16+F17+F18</f>
-        <v>84716.5421632999</v>
+        <v>85956.5915130662</v>
       </c>
       <c r="G19" s="0" t="n">
         <f aca="false">G15+G16+G17+G18</f>
-        <v>136081.200936984</v>
+        <v>137420.454234732</v>
       </c>
       <c r="H19" s="0" t="n">
         <f aca="false">H15+H16+H17+H18</f>
-        <v>178129.018102643</v>
+        <v>178845.518616938</v>
       </c>
       <c r="I19" s="0" t="n">
         <f aca="false">I15+I16+I17+I18</f>
@@ -6291,7 +6318,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="C20" s="0" t="n">
         <f aca="false">1/(1+$B$27/100)^C4</f>
@@ -6336,31 +6363,31 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="C21" s="0" t="n">
         <f aca="false">C19*C20</f>
-        <v>-96583.2645</v>
+        <v>-105218.94462</v>
       </c>
       <c r="D21" s="0" t="n">
         <f aca="false">D19*D20</f>
-        <v>-37733.6775317355</v>
+        <v>-46447.8638346446</v>
       </c>
       <c r="E21" s="0" t="n">
         <f aca="false">E19*E20</f>
-        <v>13873.901877</v>
+        <v>15156.0130196529</v>
       </c>
       <c r="F21" s="0" t="n">
         <f aca="false">F19*F20</f>
-        <v>57862.5381895361</v>
+        <v>58709.5085807432</v>
       </c>
       <c r="G21" s="0" t="n">
         <f aca="false">G19*G20</f>
-        <v>84495.7193292708</v>
+        <v>85327.2902588196</v>
       </c>
       <c r="H21" s="0" t="n">
         <f aca="false">H19*H20</f>
-        <v>100549.18690502</v>
+        <v>100953.632766209</v>
       </c>
       <c r="I21" s="0" t="n">
         <f aca="false">I19*I20</f>
@@ -6381,7 +6408,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C23" s="4" t="n">
         <f aca="false">Assumptions!C44</f>
@@ -6426,7 +6453,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C24" s="0" t="n">
         <f aca="false">-C6*C23/100</f>
@@ -6471,12 +6498,12 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B27" s="4" t="n">
         <f aca="false">Assumptions!$B$48</f>
@@ -6485,7 +6512,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B28" s="4" t="n">
         <f aca="false">Assumptions!$B$49</f>
@@ -6494,7 +6521,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B29" s="4" t="n">
         <f aca="false">Assumptions!$B$50</f>
@@ -6503,16 +6530,16 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="B30" s="0" t="n">
         <f aca="false">SUM(C21:L21)</f>
-        <v>540341.263319145</v>
+        <v>526356.495220835</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="B31" s="0" t="n">
         <f aca="false">L19</f>
@@ -6521,7 +6548,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="B32" s="0" t="n">
         <f aca="false">IF(B27&gt;B28,B31*(1+B28/100)/((B27-B28)/100),B31*B29)</f>
@@ -6530,7 +6557,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B33" s="0" t="n">
         <f aca="false">B31*B29</f>
@@ -6539,7 +6566,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="B34" s="0" t="n">
         <f aca="false">MAX(0,MIN(B32,B33))</f>
@@ -6548,7 +6575,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B35" s="0" t="n">
         <f aca="false">B34/(1+B27/100)^L4</f>
@@ -6557,52 +6584,52 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="B36" s="0" t="n">
         <f aca="false">B30+B35</f>
-        <v>2029095.93063561</v>
+        <v>2015111.16253729</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="B37" s="0" t="n">
         <f aca="false">B36+Assumptions!$B$5-Assumptions!$B$4</f>
-        <v>2448901.93063561</v>
+        <v>2480802.16253729</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="B38" s="0" t="n">
         <f aca="false">B37/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>149.569534084258</v>
+        <v>145.499777427439</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="B39" s="4" t="n">
         <f aca="false">B38/Assumptions!$B$2-1</f>
-        <v>0.442329161853986</v>
+        <v>0.432084423498419</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B41" s="0" t="n">
         <f aca="false">SUMPRODUCT(-C10:L10/(1+$B$27/100)^C4:L4)</f>
-        <v>133641.651535869</v>
+        <v>125387.187344129</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="B42" s="0" t="n">
         <f aca="false">IF(B27&gt;B28,-L10*(1+B28/100)/((B27-B28)/100),-L10*20)/(1+B27/100)^L4</f>
@@ -6611,16 +6638,16 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B43" s="0" t="n">
         <f aca="false">(B37+B41+B42)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>167.782140458831</v>
+        <v>162.504875120821</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B45" s="4" t="n">
         <f aca="false">Assumptions!$B$6</f>
@@ -6629,7 +6656,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="0" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="B46" s="0" t="n">
         <f aca="false">MAX(0,MIN(IF(B45&gt;B28,B31*(1+B28/100)/((B45-B28)/100),B31*B29),B31*B29))</f>
@@ -6638,11 +6665,11 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="B47" s="0" t="n">
         <f aca="false">(SUMPRODUCT(C19:L19/(1+B45/100)^C4:L4)+B46/(1+B45/100)^L4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>82.935910074753</v>
+        <v>81.5455022419468</v>
       </c>
     </row>
   </sheetData>
@@ -6669,40 +6696,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="B4" s="4" t="n">
         <f aca="false">DCF_Bear!$B$38</f>
-        <v>48.3307814076745</v>
+        <v>48.3183494075388</v>
       </c>
       <c r="C4" s="0" t="n">
         <f aca="false">B4/Assumptions!$B$2-1</f>
-        <v>-0.533936534159359</v>
+        <v>-0.524425694807689</v>
       </c>
       <c r="D4" s="4" t="n">
         <f aca="false">Assumptions!$B$24</f>
@@ -6710,24 +6737,24 @@
       </c>
       <c r="E4" s="4" t="n">
         <f aca="false">DCF_Bear!$B$43</f>
-        <v>60.3368973528279</v>
+        <v>59.4246144865056</v>
       </c>
       <c r="F4" s="4" t="n">
         <f aca="false">DCF_Bear!$B$47</f>
-        <v>30.5373932118357</v>
+        <v>31.2654915572399</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="B5" s="4" t="n">
         <f aca="false">DCF_Base!$B$38</f>
-        <v>97.8004930493348</v>
+        <v>95.8027665061798</v>
       </c>
       <c r="C5" s="0" t="n">
         <f aca="false">B5/Assumptions!$B$2-1</f>
-        <v>-0.0568901345290768</v>
+        <v>-0.0570593847816948</v>
       </c>
       <c r="D5" s="4" t="n">
         <f aca="false">Assumptions!$B$38</f>
@@ -6735,24 +6762,24 @@
       </c>
       <c r="E5" s="4" t="n">
         <f aca="false">DCF_Base!$B$43</f>
-        <v>113.887994416978</v>
+        <v>110.787799467257</v>
       </c>
       <c r="F5" s="4" t="n">
         <f aca="false">DCF_Base!$B$47</f>
-        <v>53.410096657993</v>
+        <v>53.2082823457069</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="B6" s="4" t="n">
         <f aca="false">DCF_Bull!$B$38</f>
-        <v>149.569534084258</v>
+        <v>145.499777427439</v>
       </c>
       <c r="C6" s="0" t="n">
         <f aca="false">B6/Assumptions!$B$2-1</f>
-        <v>0.442329161853986</v>
+        <v>0.432084423498419</v>
       </c>
       <c r="D6" s="4" t="n">
         <f aca="false">Assumptions!$B$52</f>
@@ -6760,73 +6787,73 @@
       </c>
       <c r="E6" s="4" t="n">
         <f aca="false">DCF_Bull!$B$43</f>
-        <v>167.782140458831</v>
+        <v>162.504875120821</v>
       </c>
       <c r="F6" s="4" t="n">
         <f aca="false">DCF_Bull!$B$47</f>
-        <v>82.935910074753</v>
+        <v>81.5455022419468</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="B8" s="0" t="n">
         <f aca="false">SUMPRODUCT(B4:B6,D4:D6)</f>
-        <v>93.3133877638214</v>
+        <v>91.4968435608394</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B9" s="0" t="n">
         <f aca="false">SUMPRODUCT(E4:E6,D4:D6)</f>
-        <v>108.601494506104</v>
+        <v>105.722259103744</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="B10" s="0" t="n">
         <f aca="false">1-Assumptions!$B$2/B8</f>
-        <v>-0.111308918099377</v>
+        <v>-0.110420819407203</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="B11" s="0" t="n">
         <f aca="false">IF(ABS(B9-B8)&gt;0.01*ABS(B8),(Assumptions!$B$2-B8)/(B9-B8)*100,"n/a")</f>
-        <v>67.939166119585</v>
+        <v>71.021872146292</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="B12" s="0" t="n">
         <f aca="false">SUMPRODUCT(F4:F6,D4:D6)</f>
-        <v>52.4534483074978</v>
+        <v>52.2928890884148</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="B15" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$C$15/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($C$15&gt;DCF_Base!$B$28,DCF_Base!$L$19*(1+DCF_Base!$B$28/100)/(($C$15-DCF_Base!$B$28)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$C$15/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>106.510279793465</v>
+        <v>104.160055838452</v>
       </c>
       <c r="C15" s="3" t="n">
         <v>9</v>
@@ -6834,11 +6861,11 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="B16" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$C$16/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($C$16&gt;DCF_Base!$B$28,DCF_Base!$L$19*(1+DCF_Base!$B$28/100)/(($C$16-DCF_Base!$B$28)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$C$16/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>97.8004930493348</v>
+        <v>95.8027665061798</v>
       </c>
       <c r="C16" s="3" t="n">
         <v>10</v>
@@ -6846,11 +6873,11 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="B17" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$C$17/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($C$17&gt;DCF_Base!$B$28,DCF_Base!$L$19*(1+DCF_Base!$B$28/100)/(($C$17-DCF_Base!$B$28)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$C$17/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>84.0574160790209</v>
+        <v>82.612113793784</v>
       </c>
       <c r="C17" s="3" t="n">
         <v>11</v>
@@ -6858,11 +6885,11 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="B18" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$C$18/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($C$18&gt;DCF_Base!$B$28,DCF_Base!$L$19*(1+DCF_Base!$B$28/100)/(($C$18-DCF_Base!$B$28)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$C$18/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>73.5698194045633</v>
+        <v>72.5476400407416</v>
       </c>
       <c r="C18" s="3" t="n">
         <v>12</v>
@@ -6870,11 +6897,11 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="B19" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$C$19/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($C$19&gt;DCF_Base!$B$28,DCF_Base!$L$19*(1+DCF_Base!$B$28/100)/(($C$19-DCF_Base!$B$28)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$C$19/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>53.410096657993</v>
+        <v>53.2082823457069</v>
       </c>
       <c r="C19" s="3" t="n">
         <v>15</v>
@@ -6882,7 +6909,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6908,23 +6935,23 @@
       </c>
       <c r="B23" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$23/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$23&gt;$B$22,DCF_Base!$L$19*(1+$B$22/100)/(($A$23-$B$22)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$23/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>114.803642613134</v>
+        <v>112.117481472561</v>
       </c>
       <c r="C23" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$23/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$23&gt;$C$22,DCF_Base!$L$19*(1+$C$22/100)/(($A$23-$C$22)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$23/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>114.803642613134</v>
+        <v>112.117481472561</v>
       </c>
       <c r="D23" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$23/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$23&gt;$D$22,DCF_Base!$L$19*(1+$D$22/100)/(($A$23-$D$22)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$23/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>114.803642613134</v>
+        <v>112.117481472561</v>
       </c>
       <c r="E23" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$23/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$23&gt;$E$22,DCF_Base!$L$19*(1+$E$22/100)/(($A$23-$E$22)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$23/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>114.803642613134</v>
+        <v>112.117481472561</v>
       </c>
       <c r="F23" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$23/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$23&gt;$F$22,DCF_Base!$L$19*(1+$F$22/100)/(($A$23-$F$22)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$23/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>114.803642613134</v>
+        <v>112.117481472561</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6933,23 +6960,23 @@
       </c>
       <c r="B24" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$24/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$24&gt;$B$22,DCF_Base!$L$19*(1+$B$22/100)/(($A$24-$B$22)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$24/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>104.544721035509</v>
+        <v>102.27256661374</v>
       </c>
       <c r="C24" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$24/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$24&gt;$C$22,DCF_Base!$L$19*(1+$C$22/100)/(($A$24-$C$22)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$24/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>106.510279793465</v>
+        <v>104.160055838452</v>
       </c>
       <c r="D24" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$24/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$24&gt;$D$22,DCF_Base!$L$19*(1+$D$22/100)/(($A$24-$D$22)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$24/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>106.510279793465</v>
+        <v>104.160055838452</v>
       </c>
       <c r="E24" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$24/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$24&gt;$E$22,DCF_Base!$L$19*(1+$E$22/100)/(($A$24-$E$22)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$24/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>106.510279793465</v>
+        <v>104.160055838452</v>
       </c>
       <c r="F24" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$24/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$24&gt;$F$22,DCF_Base!$L$19*(1+$F$22/100)/(($A$24-$F$22)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$24/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>106.510279793465</v>
+        <v>104.160055838452</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6958,23 +6985,23 @@
       </c>
       <c r="B25" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$25/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$25&gt;$B$22,DCF_Base!$L$19*(1+$B$22/100)/(($A$25-$B$22)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$25/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>89.5779604813901</v>
+        <v>87.9068226383051</v>
       </c>
       <c r="C25" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$25/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$25&gt;$C$22,DCF_Base!$L$19*(1+$C$22/100)/(($A$25-$C$22)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$25/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>93.415142346431</v>
+        <v>91.5915964433133</v>
       </c>
       <c r="D25" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$25/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$25&gt;$D$22,DCF_Base!$L$19*(1+$D$22/100)/(($A$25-$D$22)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$25/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>97.8004930493348</v>
+        <v>95.8027665061798</v>
       </c>
       <c r="E25" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$25/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$25&gt;$E$22,DCF_Base!$L$19*(1+$E$22/100)/(($A$25-$E$22)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$25/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>98.9964977864903</v>
+        <v>96.9512674324162</v>
       </c>
       <c r="F25" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$25/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$25&gt;$F$22,DCF_Base!$L$19*(1+$F$22/100)/(($A$25-$F$22)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$25/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>98.9964977864903</v>
+        <v>96.9512674324162</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6983,23 +7010,23 @@
       </c>
       <c r="B26" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$26/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$26&gt;$B$22,DCF_Base!$L$19*(1+$B$22/100)/(($A$26-$B$22)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$26/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>78.162352542627</v>
+        <v>76.9511948012118</v>
       </c>
       <c r="C26" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$26/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$26&gt;$C$22,DCF_Base!$L$19*(1+$C$22/100)/(($A$26-$C$22)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$26/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>80.9365000891653</v>
+        <v>79.6151566800693</v>
       </c>
       <c r="D26" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$26/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$26&gt;$D$22,DCF_Base!$L$19*(1+$D$22/100)/(($A$26-$D$22)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$26/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>84.0574160790209</v>
+        <v>82.612113793784</v>
       </c>
       <c r="E26" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$26/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$26&gt;$E$22,DCF_Base!$L$19*(1+$E$22/100)/(($A$26-$E$22)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$26/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>87.5944542008572</v>
+        <v>86.0086651893274</v>
       </c>
       <c r="F26" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$26/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$26&gt;$F$22,DCF_Base!$L$19*(1+$F$22/100)/(($A$26-$F$22)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$26/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>91.636783482956</v>
+        <v>89.8904382128055</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7008,23 +7035,23 @@
       </c>
       <c r="B27" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$27/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$27&gt;$B$22,DCF_Base!$L$19*(1+$B$22/100)/(($A$27-$B$22)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$27/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>69.2194805886355</v>
+        <v>68.3700912365308</v>
       </c>
       <c r="C27" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$27/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$27&gt;$C$22,DCF_Base!$L$19*(1+$C$22/100)/(($A$27-$C$22)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$27/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>71.2801673961803</v>
+        <v>70.3489301437885</v>
       </c>
       <c r="D27" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$27/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$27&gt;$D$22,DCF_Base!$L$19*(1+$D$22/100)/(($A$27-$D$22)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$27/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>73.5698194045633</v>
+        <v>72.5476400407416</v>
       </c>
       <c r="E27" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$27/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$27&gt;$E$22,DCF_Base!$L$19*(1+$E$22/100)/(($A$27-$E$22)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$27/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>76.1288422374619</v>
+        <v>75.0050216902774</v>
       </c>
       <c r="F27" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$27/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$27&gt;$F$22,DCF_Base!$L$19*(1+$F$22/100)/(($A$27-$F$22)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$27/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>79.0077429244729</v>
+        <v>77.7695760460051</v>
       </c>
     </row>
   </sheetData>

</xml_diff>